<commit_message>
Analizador sintactico ahora si...
</commit_message>
<xml_diff>
--- a/App/models/Tabla.xlsx
+++ b/App/models/Tabla.xlsx
@@ -5,22 +5,23 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marty\PyCharmProjects\Lenguaje y Automatas I\App\models\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF10A721-E2A3-4AB3-9387-52C3FB59A2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{919CC425-EF02-41CA-A1A6-A50D9F797E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="98">
   <si>
     <t>No-Terminal</t>
   </si>
@@ -160,21 +161,6 @@
     <t>list-arg</t>
   </si>
   <si>
-    <t>id siglist</t>
-  </si>
-  <si>
-    <t>idp siglist</t>
-  </si>
-  <si>
-    <t>num siglist</t>
-  </si>
-  <si>
-    <t>litcad siglist</t>
-  </si>
-  <si>
-    <t>litcar siglist</t>
-  </si>
-  <si>
     <t>siglist</t>
   </si>
   <si>
@@ -200,9 +186,6 @@
   </si>
   <si>
     <t>llamada</t>
-  </si>
-  <si>
-    <t>id = ( L )</t>
   </si>
   <si>
     <t>L</t>
@@ -452,7 +435,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -767,16 +750,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AQ19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.1796875" customWidth="1"/>
-    <col min="2" max="3" width="10.90625" customWidth="1"/>
-    <col min="24" max="24" width="16.26953125" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="2" max="3" width="10.88671875" customWidth="1"/>
+    <col min="24" max="24" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="27.5" customHeight="1" thickBot="1">
+    <row r="1" spans="1:43" ht="27.45" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -895,7 +878,7 @@
         <v>38</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="AO1" s="1" t="s">
         <v>39</v>
@@ -907,135 +890,135 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="30.5" customHeight="1" thickBot="1">
+    <row r="2" spans="1:43" ht="30.45" customHeight="1" thickBot="1">
       <c r="A2" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="AC2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AN2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AP2" s="2" t="s">
         <v>40</v>
       </c>
       <c r="AQ2" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:43" ht="40.5" customHeight="1" thickBot="1">
@@ -1043,121 +1026,121 @@
         <v>43</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC3" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM3" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN3" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO3" s="2" t="s">
         <v>44</v>
@@ -1174,347 +1157,347 @@
         <v>45</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="V4" s="2" t="s">
         <v>44</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="Y4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="Z4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="AA4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="AB4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AN4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AP4" s="2" t="s">
         <v>40</v>
       </c>
       <c r="AQ4" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="18.5" customHeight="1" thickBot="1">
+    <row r="5" spans="1:43" ht="18.45" customHeight="1" thickBot="1">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="X5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AN5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AP5" s="2" t="s">
         <v>40</v>
       </c>
       <c r="AQ5" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:43" ht="30.5" customHeight="1" thickBot="1">
+    <row r="6" spans="1:43" ht="30.45" customHeight="1" thickBot="1">
       <c r="A6" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="U6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="V6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="AB6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC6" s="2" t="s">
         <v>44</v>
@@ -1523,37 +1506,37 @@
         <v>44</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI6" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AJ6" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AK6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM6" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN6" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO6" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AP6" s="3" t="s">
         <v>40</v>
@@ -1562,141 +1545,141 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="30.5" customHeight="1" thickBot="1">
+    <row r="7" spans="1:43" ht="30.45" customHeight="1" thickBot="1">
       <c r="A7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="X7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI7" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="AJ7" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="AK7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ7" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" ht="20.55" customHeight="1" thickBot="1">
+      <c r="A8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="W7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="X7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AA7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AC7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AD7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AE7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AF7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AG7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AH7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AI7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ7" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="AK7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AM7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AO7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AP7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ7" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:43" ht="20.5" customHeight="1" thickBot="1">
-      <c r="A8" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="B8" s="2" t="s">
         <v>44</v>
       </c>
@@ -1770,7 +1753,7 @@
         <v>44</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA8" s="2" t="s">
         <v>44</v>
@@ -1803,16 +1786,16 @@
         <v>44</v>
       </c>
       <c r="AK8" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="AL8" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM8" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN8" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO8" s="2" t="s">
         <v>44</v>
@@ -1826,94 +1809,94 @@
     </row>
     <row r="9" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A9" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE9" s="3" t="s">
         <v>30</v>
@@ -1928,153 +1911,153 @@
         <v>33</v>
       </c>
       <c r="AI9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AN9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AP9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AQ9" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A10" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM10" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO10" s="2" t="s">
         <v>44</v>
@@ -2083,242 +2066,242 @@
         <v>44</v>
       </c>
       <c r="AQ10" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A11" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="V11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="Z11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="AA11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM11" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AN11" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AP11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="AQ11" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A12" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W12" s="2" t="s">
         <v>44</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI12" s="2" t="s">
         <v>44</v>
@@ -2327,16 +2310,16 @@
         <v>44</v>
       </c>
       <c r="AK12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM12" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN12" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO12" s="2" t="s">
         <v>44</v>
@@ -2350,190 +2333,190 @@
     </row>
     <row r="13" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A13" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="H13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="U13" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="I13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="O13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="R13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="S13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="T13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="U13" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="V13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="X13" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="X13" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="Y13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="Z13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="AA13" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="AB13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM13" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AN13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AP13" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AQ13" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="R14" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q14" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="R14" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="S14" s="2" t="s">
         <v>44</v>
       </c>
@@ -2541,46 +2524,46 @@
         <v>44</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W14" s="2" t="s">
         <v>44</v>
       </c>
       <c r="X14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI14" s="2" t="s">
         <v>44</v>
@@ -2589,16 +2572,16 @@
         <v>44</v>
       </c>
       <c r="AK14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM14" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN14" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO14" s="2" t="s">
         <v>44</v>
@@ -2612,171 +2595,171 @@
     </row>
     <row r="15" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A15" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="V15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="X15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="Z15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="AA15" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="AB15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM15" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AN15" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO15" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AP15" s="1" t="s">
         <v>40</v>
       </c>
       <c r="AQ15" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A16" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>44</v>
@@ -2803,46 +2786,46 @@
         <v>44</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W16" s="2" t="s">
         <v>44</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI16" s="2" t="s">
         <v>44</v>
@@ -2851,16 +2834,16 @@
         <v>44</v>
       </c>
       <c r="AK16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM16" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN16" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO16" s="2" t="s">
         <v>44</v>
@@ -2874,156 +2857,156 @@
     </row>
     <row r="17" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A17" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="Z17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="AA17" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="AB17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AN17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AP17" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AQ17" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A18" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>44</v>
@@ -3035,10 +3018,10 @@
         <v>44</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>44</v>
@@ -3065,46 +3048,46 @@
         <v>44</v>
       </c>
       <c r="U18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>44</v>
       </c>
       <c r="X18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Y18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Z18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AA18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI18" s="2" t="s">
         <v>44</v>
@@ -3113,16 +3096,16 @@
         <v>44</v>
       </c>
       <c r="AK18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM18" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AN18" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO18" s="2" t="s">
         <v>44</v>
@@ -3136,13 +3119,13 @@
     </row>
     <row r="19" spans="1:43" ht="15" customHeight="1" thickBot="1">
       <c r="A19" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>3</v>
@@ -3154,55 +3137,55 @@
         <v>5</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U19" s="3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="V19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="W19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X19" s="3" t="s">
         <v>23</v>
@@ -3211,58 +3194,58 @@
         <v>24</v>
       </c>
       <c r="Z19" s="3" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AA19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AB19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AC19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AD19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AE19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AF19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AG19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AH19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AI19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AJ19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AK19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AL19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AM19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AN19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AO19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="AP19" s="4" t="s">
         <v>40</v>
       </c>
       <c r="AQ19" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>